<commit_message>
Consolidate FullVision v2 cleanup
</commit_message>
<xml_diff>
--- a/fullvision-documentation-inventory.xlsx
+++ b/fullvision-documentation-inventory.xlsx
@@ -1291,12 +1291,12 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>docs/backend-design/TASKS.md</t>
+          <t>codex.md</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>801 lines</t>
+          <t>current</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1306,12 +1306,12 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Task queue for UI/ops follow-ups derived from the design doc set</t>
+          <t>Only active repo work list; consolidates open operational, platform, validation, deferred, and external items</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Historical cutover task retained as completed record; branch target is now main</t>
+          <t>Canonical work queue after docs cleanup (Apr 22 2026)</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>current</t>
+          <t>(deleted)</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -2634,10 +2634,14 @@
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Post-reconciliation backlog: quota, key rotation, e2e, rubric persistence, and follow-up work</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr"/>
+          <t>Former post-reconciliation backlog</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Historical reference only; unresolved items were consolidated into codex.md</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -2660,7 +2664,7 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>current</t>
+          <t>(deleted)</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -2670,10 +2674,14 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>UI-v1 backlog and shipped Tier-A work summary</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr"/>
+          <t>Former UI-v1 backlog and shipped Tier-A summary</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Historical reference only; unresolved items were consolidated into codex.md</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">

</xml_diff>